<commit_message>
Upload old materials, comment codes
Add kicad files for v2 build, add/comment on arduino codes for both versions, add a continuous version for v5. Finish commenting matlab codes and add calibration data for the 5 stations.
</commit_message>
<xml_diff>
--- a/KiCAD_files/weather_station_v5/Weather_station_v5_components_unsoldered.xlsx
+++ b/KiCAD_files/weather_station_v5/Weather_station_v5_components_unsoldered.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shiel\Documents\Github\low-power-weather-station\KiCAD_files\weather_station_lowpower\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shiel\Documents\Github\low-power-weather-station\KiCAD_files\weather_station_v5\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AFDC9EA-7147-4F5E-8815-D4AA832672A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F267C021-762C-4D26-A129-E33A6D668369}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2580" yWindow="1776" windowWidth="15768" windowHeight="9594" xr2:uid="{F9B17DE7-B4AA-4BE7-856E-F3D66462765B}"/>
+    <workbookView xWindow="876" yWindow="336" windowWidth="22116" windowHeight="12738" xr2:uid="{F9B17DE7-B4AA-4BE7-856E-F3D66462765B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>